<commit_message>
Actualización automática ERP - Pedidos Pendientes - 11/08/2026 14:28:50
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE239974-01D9-4137-80D8-2A9801E25BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{705382A6-AA0B-4317-8414-BDDB70B95321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{371C2092-AB7E-472A-9A96-4391D667F6EC}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A52CF64B-8E78-4B94-85F3-B18295D69920}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -5129,7 +5129,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39865B90-8C8C-4105-B70C-1053E0788781}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24F3B0F-F821-4771-8A23-CDE584A10446}">
   <dimension ref="A1:BI342"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 12/08/2026 08:17:23
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF4D0130-B808-49E8-819C-529846ACB687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A8A5140-1B1C-4D3E-A1D3-36B4B855B09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F96C1EEB-851C-4DA8-AC26-A05F5270D43C}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{091230EA-0D29-454D-8790-FEA0BA18E252}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -5465,7 +5465,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EB2C087-B9E7-4983-9AF2-3340BB4FB941}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2B3ADE6-0EDA-4416-A865-377757CC71EE}">
   <dimension ref="A1:BI385"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 22/08/2026 11:53:09
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B004F0FF-F182-4372-8631-D56DC5280F14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{57FFEC94-F38E-4C16-B86B-96BE631EA39B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{23D57EE4-CDC4-44CD-85C2-33374AE16F9D}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0BB7660C-43E8-4F6F-8587-3AA9A0B499CC}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4571,7 +4571,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21FA490-FB56-4567-9B00-F6A2FEA0BB57}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B601BAB-80F2-45E1-916B-91A6D70FEE5A}">
   <dimension ref="A1:BI327"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 24/08/2026 06:06:29
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57FFEC94-F38E-4C16-B86B-96BE631EA39B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A4F7E726-6B0B-4921-9EA4-397B224423AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{0BB7660C-43E8-4F6F-8587-3AA9A0B499CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{61361E66-B3D2-4A28-951A-D55B7AFA8C3B}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4571,7 +4571,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B601BAB-80F2-45E1-916B-91A6D70FEE5A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9CDCDFC-A533-440C-8895-B6AA0BBC43F1}">
   <dimension ref="A1:BI327"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -4777,7 +4777,7 @@
         <v>64</v>
       </c>
       <c r="F2">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G2">
         <v>11</v>
@@ -4962,10 +4962,10 @@
         <v>89</v>
       </c>
       <c r="F3">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G3">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="H3" t="s">
         <v>90</v>
@@ -5147,7 +5147,7 @@
         <v>108</v>
       </c>
       <c r="F4">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -5332,10 +5332,10 @@
         <v>120</v>
       </c>
       <c r="F5">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="G5">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H5" t="s">
         <v>121</v>
@@ -5517,10 +5517,10 @@
         <v>134</v>
       </c>
       <c r="F6">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G6">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H6" t="s">
         <v>135</v>
@@ -5702,10 +5702,10 @@
         <v>146</v>
       </c>
       <c r="F7">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G7">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H7" t="s">
         <v>147</v>
@@ -5887,10 +5887,10 @@
         <v>154</v>
       </c>
       <c r="F8">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G8">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H8" t="s">
         <v>155</v>
@@ -6072,7 +6072,7 @@
         <v>154</v>
       </c>
       <c r="F9">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G9">
         <v>6</v>
@@ -6257,10 +6257,10 @@
         <v>154</v>
       </c>
       <c r="F10">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G10">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H10" t="s">
         <v>168</v>
@@ -6442,10 +6442,10 @@
         <v>154</v>
       </c>
       <c r="F11">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G11">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H11" t="s">
         <v>176</v>
@@ -6627,10 +6627,10 @@
         <v>193</v>
       </c>
       <c r="F12">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G12">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H12" t="s">
         <v>194</v>
@@ -6812,7 +6812,7 @@
         <v>205</v>
       </c>
       <c r="F13">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G13">
         <v>7</v>
@@ -6997,10 +6997,10 @@
         <v>204</v>
       </c>
       <c r="F14">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G14">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H14" t="s">
         <v>212</v>
@@ -7182,10 +7182,10 @@
         <v>216</v>
       </c>
       <c r="F15">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G15">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H15" t="s">
         <v>217</v>
@@ -7367,7 +7367,7 @@
         <v>225</v>
       </c>
       <c r="F16">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G16">
         <v>8</v>
@@ -7552,10 +7552,10 @@
         <v>231</v>
       </c>
       <c r="F17">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G17">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H17" t="s">
         <v>232</v>
@@ -7737,10 +7737,10 @@
         <v>231</v>
       </c>
       <c r="F18">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G18">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H18" t="s">
         <v>240</v>
@@ -7922,10 +7922,10 @@
         <v>248</v>
       </c>
       <c r="F19">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G19">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H19" t="s">
         <v>249</v>
@@ -8107,10 +8107,10 @@
         <v>247</v>
       </c>
       <c r="F20">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G20">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H20" t="s">
         <v>253</v>
@@ -8292,7 +8292,7 @@
         <v>261</v>
       </c>
       <c r="F21">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G21">
         <v>4</v>
@@ -8477,10 +8477,10 @@
         <v>274</v>
       </c>
       <c r="F22">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G22">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H22" t="s">
         <v>275</v>
@@ -8662,10 +8662,10 @@
         <v>274</v>
       </c>
       <c r="F23">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G23">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H23" t="s">
         <v>281</v>
@@ -8847,7 +8847,7 @@
         <v>288</v>
       </c>
       <c r="F24">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -9032,10 +9032,10 @@
         <v>288</v>
       </c>
       <c r="F25">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G25">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H25" t="s">
         <v>295</v>
@@ -9217,10 +9217,10 @@
         <v>288</v>
       </c>
       <c r="F26">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G26">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H26" t="s">
         <v>299</v>
@@ -9402,10 +9402,10 @@
         <v>304</v>
       </c>
       <c r="F27">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G27">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H27" t="s">
         <v>305</v>
@@ -9587,10 +9587,10 @@
         <v>303</v>
       </c>
       <c r="F28">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G28">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H28" t="s">
         <v>312</v>
@@ -9772,10 +9772,10 @@
         <v>303</v>
       </c>
       <c r="F29">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G29">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H29" t="s">
         <v>317</v>
@@ -9957,10 +9957,10 @@
         <v>304</v>
       </c>
       <c r="F30">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G30">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H30" t="s">
         <v>323</v>
@@ -10142,10 +10142,10 @@
         <v>330</v>
       </c>
       <c r="F31">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G31">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H31" t="s">
         <v>331</v>
@@ -10327,10 +10327,10 @@
         <v>330</v>
       </c>
       <c r="F32">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G32">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H32" t="s">
         <v>336</v>
@@ -10512,10 +10512,10 @@
         <v>330</v>
       </c>
       <c r="F33">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G33">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H33" t="s">
         <v>341</v>
@@ -10697,10 +10697,10 @@
         <v>330</v>
       </c>
       <c r="F34">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G34">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H34" t="s">
         <v>349</v>
@@ -10882,10 +10882,10 @@
         <v>355</v>
       </c>
       <c r="F35">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G35">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H35" t="s">
         <v>356</v>
@@ -11067,10 +11067,10 @@
         <v>363</v>
       </c>
       <c r="F36">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G36">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H36" t="s">
         <v>364</v>
@@ -11252,10 +11252,10 @@
         <v>363</v>
       </c>
       <c r="F37">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G37">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H37" t="s">
         <v>368</v>
@@ -11437,10 +11437,10 @@
         <v>372</v>
       </c>
       <c r="F38">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G38">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H38" t="s">
         <v>336</v>
@@ -11622,10 +11622,10 @@
         <v>372</v>
       </c>
       <c r="F39">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G39">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H39" t="s">
         <v>376</v>
@@ -11807,10 +11807,10 @@
         <v>372</v>
       </c>
       <c r="F40">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G40">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H40" t="s">
         <v>90</v>
@@ -11992,10 +11992,10 @@
         <v>389</v>
       </c>
       <c r="F41">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G41">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H41" t="s">
         <v>323</v>
@@ -12177,10 +12177,10 @@
         <v>389</v>
       </c>
       <c r="F42">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G42">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H42" t="s">
         <v>391</v>
@@ -12362,10 +12362,10 @@
         <v>398</v>
       </c>
       <c r="F43">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G43">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H43" t="s">
         <v>399</v>
@@ -12547,10 +12547,10 @@
         <v>398</v>
       </c>
       <c r="F44">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G44">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H44" t="s">
         <v>407</v>
@@ -12732,10 +12732,10 @@
         <v>398</v>
       </c>
       <c r="F45">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G45">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H45" t="s">
         <v>413</v>
@@ -12917,10 +12917,10 @@
         <v>420</v>
       </c>
       <c r="F46">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G46">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H46" t="s">
         <v>421</v>
@@ -13102,10 +13102,10 @@
         <v>420</v>
       </c>
       <c r="F47">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G47">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H47" t="s">
         <v>427</v>
@@ -13287,10 +13287,10 @@
         <v>432</v>
       </c>
       <c r="F48">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G48">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H48" t="s">
         <v>391</v>
@@ -13472,10 +13472,10 @@
         <v>432</v>
       </c>
       <c r="F49">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G49">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H49" t="s">
         <v>295</v>
@@ -13657,10 +13657,10 @@
         <v>432</v>
       </c>
       <c r="F50">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G50">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H50" t="s">
         <v>295</v>
@@ -13842,10 +13842,10 @@
         <v>442</v>
       </c>
       <c r="F51">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G51">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="H51" t="s">
         <v>443</v>
@@ -14027,10 +14027,10 @@
         <v>454</v>
       </c>
       <c r="F52">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G52">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H52" t="s">
         <v>455</v>
@@ -14212,10 +14212,10 @@
         <v>454</v>
       </c>
       <c r="F53">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G53">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H53" t="s">
         <v>459</v>
@@ -14397,10 +14397,10 @@
         <v>454</v>
       </c>
       <c r="F54">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G54">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H54" t="s">
         <v>463</v>
@@ -14582,10 +14582,10 @@
         <v>454</v>
       </c>
       <c r="F55">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G55">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H55" t="s">
         <v>468</v>
@@ -14767,10 +14767,10 @@
         <v>474</v>
       </c>
       <c r="F56">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G56">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H56" t="s">
         <v>289</v>
@@ -14952,10 +14952,10 @@
         <v>474</v>
       </c>
       <c r="F57">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G57">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H57" t="s">
         <v>476</v>
@@ -15137,10 +15137,10 @@
         <v>474</v>
       </c>
       <c r="F58">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G58">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H58" t="s">
         <v>480</v>
@@ -15322,10 +15322,10 @@
         <v>483</v>
       </c>
       <c r="F59">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G59">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H59" t="s">
         <v>484</v>
@@ -15507,10 +15507,10 @@
         <v>483</v>
       </c>
       <c r="F60">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G60">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H60" t="s">
         <v>421</v>
@@ -15692,10 +15692,10 @@
         <v>483</v>
       </c>
       <c r="F61">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G61">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H61" t="s">
         <v>492</v>
@@ -15877,10 +15877,10 @@
         <v>497</v>
       </c>
       <c r="F62">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G62">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H62" t="s">
         <v>498</v>
@@ -16062,10 +16062,10 @@
         <v>503</v>
       </c>
       <c r="F63">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G63">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H63" t="s">
         <v>504</v>
@@ -16247,10 +16247,10 @@
         <v>503</v>
       </c>
       <c r="F64">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="G64">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H64" t="s">
         <v>508</v>
@@ -16432,10 +16432,10 @@
         <v>503</v>
       </c>
       <c r="F65">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G65">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H65" t="s">
         <v>514</v>
@@ -16617,10 +16617,10 @@
         <v>503</v>
       </c>
       <c r="F66">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G66">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H66" t="s">
         <v>519</v>
@@ -16802,10 +16802,10 @@
         <v>524</v>
       </c>
       <c r="F67">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G67">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H67" t="s">
         <v>525</v>
@@ -16987,10 +16987,10 @@
         <v>524</v>
       </c>
       <c r="F68">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G68">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H68" t="s">
         <v>529</v>
@@ -17172,10 +17172,10 @@
         <v>524</v>
       </c>
       <c r="F69">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G69">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H69" t="s">
         <v>535</v>
@@ -17357,10 +17357,10 @@
         <v>524</v>
       </c>
       <c r="F70">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G70">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H70" t="s">
         <v>541</v>
@@ -17542,10 +17542,10 @@
         <v>524</v>
       </c>
       <c r="F71">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G71">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H71" t="s">
         <v>541</v>
@@ -17727,10 +17727,10 @@
         <v>548</v>
       </c>
       <c r="F72">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G72">
-        <v>-11</v>
+        <v>-9</v>
       </c>
       <c r="H72" t="s">
         <v>443</v>
@@ -17912,10 +17912,10 @@
         <v>551</v>
       </c>
       <c r="F73">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G73">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H73" t="s">
         <v>455</v>
@@ -18097,10 +18097,10 @@
         <v>524</v>
       </c>
       <c r="F74">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G74">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H74" t="s">
         <v>281</v>
@@ -18282,7 +18282,7 @@
         <v>524</v>
       </c>
       <c r="F75">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G75">
         <v>6</v>
@@ -18467,10 +18467,10 @@
         <v>524</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G76">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H76" t="s">
         <v>555</v>
@@ -18652,10 +18652,10 @@
         <v>551</v>
       </c>
       <c r="F77">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G77">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H77" t="s">
         <v>560</v>
@@ -18837,10 +18837,10 @@
         <v>524</v>
       </c>
       <c r="F78">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G78">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H78" t="s">
         <v>564</v>
@@ -19022,10 +19022,10 @@
         <v>551</v>
       </c>
       <c r="F79">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G79">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H79" t="s">
         <v>232</v>
@@ -19207,10 +19207,10 @@
         <v>573</v>
       </c>
       <c r="F80">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G80">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H80" t="s">
         <v>443</v>
@@ -19392,10 +19392,10 @@
         <v>573</v>
       </c>
       <c r="F81">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G81">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H81" t="s">
         <v>443</v>
@@ -19577,10 +19577,10 @@
         <v>573</v>
       </c>
       <c r="F82">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G82">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H82" t="s">
         <v>443</v>
@@ -19762,10 +19762,10 @@
         <v>573</v>
       </c>
       <c r="F83">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G83">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H83" t="s">
         <v>443</v>
@@ -19947,10 +19947,10 @@
         <v>573</v>
       </c>
       <c r="F84">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G84">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H84" t="s">
         <v>443</v>
@@ -20132,10 +20132,10 @@
         <v>573</v>
       </c>
       <c r="F85">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G85">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H85" t="s">
         <v>443</v>
@@ -20317,10 +20317,10 @@
         <v>573</v>
       </c>
       <c r="F86">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G86">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H86" t="s">
         <v>443</v>
@@ -20502,10 +20502,10 @@
         <v>573</v>
       </c>
       <c r="F87">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G87">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H87" t="s">
         <v>443</v>
@@ -20687,10 +20687,10 @@
         <v>573</v>
       </c>
       <c r="F88">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G88">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H88" t="s">
         <v>443</v>
@@ -20872,10 +20872,10 @@
         <v>573</v>
       </c>
       <c r="F89">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G89">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H89" t="s">
         <v>443</v>
@@ -21057,10 +21057,10 @@
         <v>573</v>
       </c>
       <c r="F90">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G90">
-        <v>-12</v>
+        <v>-10</v>
       </c>
       <c r="H90" t="s">
         <v>443</v>
@@ -21242,10 +21242,10 @@
         <v>600</v>
       </c>
       <c r="F91">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G91">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H91" t="s">
         <v>601</v>
@@ -21427,10 +21427,10 @@
         <v>600</v>
       </c>
       <c r="F92">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G92">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H92" t="s">
         <v>331</v>
@@ -21612,10 +21612,10 @@
         <v>600</v>
       </c>
       <c r="F93">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G93">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H93" t="s">
         <v>608</v>
@@ -21797,10 +21797,10 @@
         <v>600</v>
       </c>
       <c r="F94">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G94">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H94" t="s">
         <v>612</v>
@@ -21982,10 +21982,10 @@
         <v>600</v>
       </c>
       <c r="F95">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G95">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H95" t="s">
         <v>616</v>
@@ -22167,10 +22167,10 @@
         <v>622</v>
       </c>
       <c r="F96">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G96">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H96" t="s">
         <v>623</v>
@@ -22352,10 +22352,10 @@
         <v>622</v>
       </c>
       <c r="F97">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G97">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H97" t="s">
         <v>161</v>
@@ -22537,10 +22537,10 @@
         <v>600</v>
       </c>
       <c r="F98">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G98">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H98" t="s">
         <v>413</v>
@@ -22722,10 +22722,10 @@
         <v>600</v>
       </c>
       <c r="F99">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G99">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H99" t="s">
         <v>631</v>
@@ -22907,7 +22907,7 @@
         <v>622</v>
       </c>
       <c r="F100">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G100">
         <v>5</v>
@@ -23092,10 +23092,10 @@
         <v>622</v>
       </c>
       <c r="F101">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G101">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H101" t="s">
         <v>637</v>
@@ -23277,10 +23277,10 @@
         <v>622</v>
       </c>
       <c r="F102">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G102">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H102" t="s">
         <v>642</v>
@@ -23462,10 +23462,10 @@
         <v>648</v>
       </c>
       <c r="F103">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G103">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H103" t="s">
         <v>649</v>
@@ -23647,10 +23647,10 @@
         <v>654</v>
       </c>
       <c r="F104">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G104">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H104" t="s">
         <v>655</v>
@@ -23832,10 +23832,10 @@
         <v>654</v>
       </c>
       <c r="F105">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G105">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H105" t="s">
         <v>601</v>
@@ -24017,10 +24017,10 @@
         <v>654</v>
       </c>
       <c r="F106">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G106">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H106" t="s">
         <v>663</v>
@@ -24202,10 +24202,10 @@
         <v>654</v>
       </c>
       <c r="F107">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G107">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H107" t="s">
         <v>109</v>
@@ -24387,10 +24387,10 @@
         <v>648</v>
       </c>
       <c r="F108">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G108">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H108" t="s">
         <v>671</v>
@@ -24572,10 +24572,10 @@
         <v>654</v>
       </c>
       <c r="F109">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G109">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H109" t="s">
         <v>161</v>
@@ -24757,10 +24757,10 @@
         <v>654</v>
       </c>
       <c r="F110">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G110">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H110" t="s">
         <v>616</v>
@@ -24942,10 +24942,10 @@
         <v>654</v>
       </c>
       <c r="F111">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G111">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H111" t="s">
         <v>391</v>
@@ -25127,10 +25127,10 @@
         <v>654</v>
       </c>
       <c r="F112">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G112">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H112" t="s">
         <v>421</v>
@@ -25312,10 +25312,10 @@
         <v>654</v>
       </c>
       <c r="F113">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G113">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H113" t="s">
         <v>427</v>
@@ -25497,10 +25497,10 @@
         <v>654</v>
       </c>
       <c r="F114">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G114">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H114" t="s">
         <v>686</v>
@@ -25682,7 +25682,7 @@
         <v>654</v>
       </c>
       <c r="F115">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G115">
         <v>2</v>
@@ -25867,7 +25867,7 @@
         <v>648</v>
       </c>
       <c r="F116">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G116">
         <v>2</v>
@@ -26052,10 +26052,10 @@
         <v>654</v>
       </c>
       <c r="F117">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G117">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H117" t="s">
         <v>700</v>
@@ -26237,10 +26237,10 @@
         <v>654</v>
       </c>
       <c r="F118">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G118">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H118" t="s">
         <v>703</v>
@@ -26422,10 +26422,10 @@
         <v>648</v>
       </c>
       <c r="F119">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G119">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H119" t="s">
         <v>707</v>
@@ -26607,10 +26607,10 @@
         <v>654</v>
       </c>
       <c r="F120">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G120">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H120" t="s">
         <v>65</v>
@@ -26792,10 +26792,10 @@
         <v>654</v>
       </c>
       <c r="F121">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G121">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H121" t="s">
         <v>492</v>
@@ -26977,10 +26977,10 @@
         <v>654</v>
       </c>
       <c r="F122">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G122">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H122" t="s">
         <v>492</v>
@@ -27162,7 +27162,7 @@
         <v>654</v>
       </c>
       <c r="F123">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G123">
         <v>2</v>
@@ -27347,10 +27347,10 @@
         <v>654</v>
       </c>
       <c r="F124">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G124">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H124" t="s">
         <v>323</v>
@@ -27532,10 +27532,10 @@
         <v>654</v>
       </c>
       <c r="F125">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G125">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H125" t="s">
         <v>724</v>
@@ -27717,10 +27717,10 @@
         <v>654</v>
       </c>
       <c r="F126">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G126">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H126" t="s">
         <v>732</v>
@@ -27902,10 +27902,10 @@
         <v>654</v>
       </c>
       <c r="F127">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G127">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H127" t="s">
         <v>740</v>
@@ -28087,10 +28087,10 @@
         <v>746</v>
       </c>
       <c r="F128">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G128">
-        <v>-17</v>
+        <v>-15</v>
       </c>
       <c r="H128" t="s">
         <v>443</v>
@@ -28272,10 +28272,10 @@
         <v>654</v>
       </c>
       <c r="F129">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G129">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H129" t="s">
         <v>413</v>
@@ -28457,10 +28457,10 @@
         <v>751</v>
       </c>
       <c r="F130">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G130">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H130" t="s">
         <v>752</v>
@@ -28642,10 +28642,10 @@
         <v>654</v>
       </c>
       <c r="F131">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G131">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H131" t="s">
         <v>757</v>
@@ -28827,10 +28827,10 @@
         <v>751</v>
       </c>
       <c r="F132">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G132">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H132" t="s">
         <v>765</v>
@@ -29012,10 +29012,10 @@
         <v>751</v>
       </c>
       <c r="F133">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G133">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H133" t="s">
         <v>769</v>
@@ -29197,10 +29197,10 @@
         <v>751</v>
       </c>
       <c r="F134">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G134">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H134" t="s">
         <v>774</v>
@@ -29382,10 +29382,10 @@
         <v>751</v>
       </c>
       <c r="F135">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G135">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H135" t="s">
         <v>686</v>
@@ -29567,10 +29567,10 @@
         <v>751</v>
       </c>
       <c r="F136">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G136">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H136" t="s">
         <v>780</v>
@@ -29752,10 +29752,10 @@
         <v>751</v>
       </c>
       <c r="F137">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G137">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H137" t="s">
         <v>780</v>
@@ -29937,10 +29937,10 @@
         <v>751</v>
       </c>
       <c r="F138">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G138">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H138" t="s">
         <v>785</v>
@@ -30122,10 +30122,10 @@
         <v>751</v>
       </c>
       <c r="F139">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G139">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H139" t="s">
         <v>789</v>
@@ -30307,10 +30307,10 @@
         <v>793</v>
       </c>
       <c r="F140">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G140">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H140" t="s">
         <v>443</v>
@@ -30492,10 +30492,10 @@
         <v>793</v>
       </c>
       <c r="F141">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G141">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H141" t="s">
         <v>443</v>
@@ -30677,10 +30677,10 @@
         <v>793</v>
       </c>
       <c r="F142">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G142">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H142" t="s">
         <v>443</v>
@@ -30862,10 +30862,10 @@
         <v>793</v>
       </c>
       <c r="F143">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G143">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H143" t="s">
         <v>443</v>
@@ -31047,10 +31047,10 @@
         <v>793</v>
       </c>
       <c r="F144">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G144">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H144" t="s">
         <v>443</v>
@@ -31232,10 +31232,10 @@
         <v>793</v>
       </c>
       <c r="F145">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G145">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H145" t="s">
         <v>443</v>
@@ -31417,10 +31417,10 @@
         <v>793</v>
       </c>
       <c r="F146">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G146">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H146" t="s">
         <v>443</v>
@@ -31602,10 +31602,10 @@
         <v>793</v>
       </c>
       <c r="F147">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G147">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H147" t="s">
         <v>443</v>
@@ -31787,10 +31787,10 @@
         <v>793</v>
       </c>
       <c r="F148">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G148">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H148" t="s">
         <v>443</v>
@@ -31972,10 +31972,10 @@
         <v>654</v>
       </c>
       <c r="F149">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G149">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H149" t="s">
         <v>707</v>
@@ -32157,10 +32157,10 @@
         <v>654</v>
       </c>
       <c r="F150">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G150">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H150" t="s">
         <v>813</v>
@@ -32342,10 +32342,10 @@
         <v>751</v>
       </c>
       <c r="F151">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G151">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H151" t="s">
         <v>821</v>
@@ -32527,10 +32527,10 @@
         <v>751</v>
       </c>
       <c r="F152">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G152">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H152" t="s">
         <v>821</v>
@@ -32712,10 +32712,10 @@
         <v>751</v>
       </c>
       <c r="F153">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G153">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H153" t="s">
         <v>623</v>
@@ -32897,10 +32897,10 @@
         <v>751</v>
       </c>
       <c r="F154">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G154">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H154" t="s">
         <v>828</v>
@@ -33082,10 +33082,10 @@
         <v>751</v>
       </c>
       <c r="F155">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G155">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H155" t="s">
         <v>833</v>
@@ -33267,10 +33267,10 @@
         <v>836</v>
       </c>
       <c r="F156">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G156">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H156" t="s">
         <v>109</v>
@@ -33452,10 +33452,10 @@
         <v>836</v>
       </c>
       <c r="F157">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G157">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H157" t="s">
         <v>838</v>
@@ -33637,10 +33637,10 @@
         <v>751</v>
       </c>
       <c r="F158">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G158">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H158" t="s">
         <v>842</v>
@@ -33822,10 +33822,10 @@
         <v>751</v>
       </c>
       <c r="F159">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G159">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H159" t="s">
         <v>299</v>
@@ -34007,10 +34007,10 @@
         <v>793</v>
       </c>
       <c r="F160">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G160">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H160" t="s">
         <v>443</v>
@@ -34192,10 +34192,10 @@
         <v>793</v>
       </c>
       <c r="F161">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G161">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H161" t="s">
         <v>443</v>
@@ -34377,10 +34377,10 @@
         <v>793</v>
       </c>
       <c r="F162">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G162">
-        <v>-18</v>
+        <v>-16</v>
       </c>
       <c r="H162" t="s">
         <v>443</v>
@@ -34562,10 +34562,10 @@
         <v>751</v>
       </c>
       <c r="F163">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G163">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H163" t="s">
         <v>856</v>
@@ -34747,10 +34747,10 @@
         <v>751</v>
       </c>
       <c r="F164">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G164">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H164" t="s">
         <v>856</v>
@@ -34932,10 +34932,10 @@
         <v>751</v>
       </c>
       <c r="F165">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G165">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H165" t="s">
         <v>90</v>
@@ -35117,10 +35117,10 @@
         <v>751</v>
       </c>
       <c r="F166">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G166">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H166" t="s">
         <v>870</v>
@@ -35302,10 +35302,10 @@
         <v>751</v>
       </c>
       <c r="F167">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G167">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H167" t="s">
         <v>877</v>
@@ -35487,10 +35487,10 @@
         <v>751</v>
       </c>
       <c r="F168">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G168">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H168" t="s">
         <v>885</v>
@@ -35672,10 +35672,10 @@
         <v>836</v>
       </c>
       <c r="F169">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G169">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H169" t="s">
         <v>889</v>
@@ -35857,10 +35857,10 @@
         <v>836</v>
       </c>
       <c r="F170">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G170">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H170" t="s">
         <v>892</v>
@@ -36042,10 +36042,10 @@
         <v>836</v>
       </c>
       <c r="F171">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G171">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H171" t="s">
         <v>663</v>
@@ -36227,10 +36227,10 @@
         <v>751</v>
       </c>
       <c r="F172">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G172">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H172" t="s">
         <v>90</v>
@@ -36412,10 +36412,10 @@
         <v>751</v>
       </c>
       <c r="F173">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G173">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H173" t="s">
         <v>904</v>
@@ -36597,10 +36597,10 @@
         <v>836</v>
       </c>
       <c r="F174">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G174">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H174" t="s">
         <v>910</v>
@@ -36782,10 +36782,10 @@
         <v>836</v>
       </c>
       <c r="F175">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G175">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H175" t="s">
         <v>217</v>
@@ -36967,10 +36967,10 @@
         <v>751</v>
       </c>
       <c r="F176">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G176">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H176" t="s">
         <v>921</v>
@@ -37152,10 +37152,10 @@
         <v>751</v>
       </c>
       <c r="F177">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G177">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H177" t="s">
         <v>921</v>
@@ -37337,10 +37337,10 @@
         <v>836</v>
       </c>
       <c r="F178">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G178">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H178" t="s">
         <v>637</v>
@@ -37522,10 +37522,10 @@
         <v>751</v>
       </c>
       <c r="F179">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G179">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H179" t="s">
         <v>519</v>
@@ -37707,10 +37707,10 @@
         <v>751</v>
       </c>
       <c r="F180">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G180">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H180" t="s">
         <v>934</v>
@@ -37892,10 +37892,10 @@
         <v>836</v>
       </c>
       <c r="F181">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G181">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H181" t="s">
         <v>937</v>
@@ -38077,10 +38077,10 @@
         <v>751</v>
       </c>
       <c r="F182">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G182">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H182" t="s">
         <v>90</v>
@@ -38262,10 +38262,10 @@
         <v>836</v>
       </c>
       <c r="F183">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G183">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H183" t="s">
         <v>217</v>
@@ -38447,10 +38447,10 @@
         <v>836</v>
       </c>
       <c r="F184">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G184">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H184" t="s">
         <v>944</v>
@@ -38632,10 +38632,10 @@
         <v>836</v>
       </c>
       <c r="F185">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G185">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H185" t="s">
         <v>947</v>
@@ -38817,10 +38817,10 @@
         <v>751</v>
       </c>
       <c r="F186">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G186">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H186" t="s">
         <v>952</v>
@@ -39002,10 +39002,10 @@
         <v>751</v>
       </c>
       <c r="F187">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G187">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H187" t="s">
         <v>958</v>
@@ -39187,10 +39187,10 @@
         <v>751</v>
       </c>
       <c r="F188">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G188">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H188" t="s">
         <v>964</v>
@@ -39372,10 +39372,10 @@
         <v>836</v>
       </c>
       <c r="F189">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G189">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H189" t="s">
         <v>226</v>
@@ -39557,10 +39557,10 @@
         <v>751</v>
       </c>
       <c r="F190">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G190">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H190" t="s">
         <v>813</v>
@@ -39742,10 +39742,10 @@
         <v>836</v>
       </c>
       <c r="F191">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G191">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H191" t="s">
         <v>226</v>
@@ -39927,10 +39927,10 @@
         <v>836</v>
       </c>
       <c r="F192">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G192">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H192" t="s">
         <v>976</v>
@@ -40112,10 +40112,10 @@
         <v>836</v>
       </c>
       <c r="F193">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G193">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H193" t="s">
         <v>980</v>
@@ -40297,10 +40297,10 @@
         <v>836</v>
       </c>
       <c r="F194">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G194">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H194" t="s">
         <v>601</v>
@@ -40482,10 +40482,10 @@
         <v>836</v>
       </c>
       <c r="F195">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G195">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H195" t="s">
         <v>986</v>
@@ -40667,10 +40667,10 @@
         <v>836</v>
       </c>
       <c r="F196">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G196">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H196" t="s">
         <v>833</v>
@@ -40852,10 +40852,10 @@
         <v>836</v>
       </c>
       <c r="F197">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G197">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H197" t="s">
         <v>992</v>
@@ -41037,10 +41037,10 @@
         <v>836</v>
       </c>
       <c r="F198">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G198">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H198" t="s">
         <v>463</v>
@@ -41222,10 +41222,10 @@
         <v>836</v>
       </c>
       <c r="F199">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G199">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H199" t="s">
         <v>463</v>
@@ -41407,10 +41407,10 @@
         <v>836</v>
       </c>
       <c r="F200">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G200">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H200" t="s">
         <v>249</v>
@@ -41592,10 +41592,10 @@
         <v>836</v>
       </c>
       <c r="F201">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G201">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H201" t="s">
         <v>1000</v>
@@ -41777,10 +41777,10 @@
         <v>836</v>
       </c>
       <c r="F202">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G202">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H202" t="s">
         <v>1004</v>
@@ -41962,10 +41962,10 @@
         <v>836</v>
       </c>
       <c r="F203">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G203">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H203" t="s">
         <v>1007</v>
@@ -42147,10 +42147,10 @@
         <v>836</v>
       </c>
       <c r="F204">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G204">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H204" t="s">
         <v>1010</v>
@@ -42332,10 +42332,10 @@
         <v>836</v>
       </c>
       <c r="F205">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G205">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H205" t="s">
         <v>1014</v>
@@ -42517,10 +42517,10 @@
         <v>836</v>
       </c>
       <c r="F206">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G206">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H206" t="s">
         <v>249</v>
@@ -42702,10 +42702,10 @@
         <v>836</v>
       </c>
       <c r="F207">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G207">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H207" t="s">
         <v>612</v>
@@ -42887,10 +42887,10 @@
         <v>836</v>
       </c>
       <c r="F208">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G208">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H208" t="s">
         <v>1022</v>
@@ -43072,10 +43072,10 @@
         <v>836</v>
       </c>
       <c r="F209">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G209">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H209" t="s">
         <v>612</v>
@@ -43257,10 +43257,10 @@
         <v>836</v>
       </c>
       <c r="F210">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G210">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H210" t="s">
         <v>1028</v>
@@ -43442,10 +43442,10 @@
         <v>836</v>
       </c>
       <c r="F211">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G211">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H211" t="s">
         <v>1022</v>
@@ -43627,10 +43627,10 @@
         <v>836</v>
       </c>
       <c r="F212">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G212">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H212" t="s">
         <v>1034</v>
@@ -43812,10 +43812,10 @@
         <v>836</v>
       </c>
       <c r="F213">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G213">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H213" t="s">
         <v>1039</v>
@@ -43997,10 +43997,10 @@
         <v>836</v>
       </c>
       <c r="F214">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G214">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H214" t="s">
         <v>90</v>
@@ -44182,10 +44182,10 @@
         <v>1048</v>
       </c>
       <c r="F215">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G215">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H215" t="s">
         <v>1049</v>
@@ -44367,10 +44367,10 @@
         <v>1048</v>
       </c>
       <c r="F216">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G216">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H216" t="s">
         <v>109</v>
@@ -44552,10 +44552,10 @@
         <v>1048</v>
       </c>
       <c r="F217">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G217">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H217" t="s">
         <v>376</v>
@@ -44737,10 +44737,10 @@
         <v>1048</v>
       </c>
       <c r="F218">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G218">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H218" t="s">
         <v>376</v>
@@ -44922,10 +44922,10 @@
         <v>1048</v>
       </c>
       <c r="F219">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G219">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H219" t="s">
         <v>1059</v>
@@ -45107,10 +45107,10 @@
         <v>836</v>
       </c>
       <c r="F220">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G220">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H220" t="s">
         <v>90</v>
@@ -45292,10 +45292,10 @@
         <v>1048</v>
       </c>
       <c r="F221">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G221">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H221" t="s">
         <v>612</v>
@@ -45477,10 +45477,10 @@
         <v>1048</v>
       </c>
       <c r="F222">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G222">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H222" t="s">
         <v>789</v>
@@ -45662,10 +45662,10 @@
         <v>1048</v>
       </c>
       <c r="F223">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G223">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H223" t="s">
         <v>1070</v>
@@ -45847,10 +45847,10 @@
         <v>1048</v>
       </c>
       <c r="F224">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G224">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H224" t="s">
         <v>1070</v>
@@ -46032,10 +46032,10 @@
         <v>1048</v>
       </c>
       <c r="F225">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G225">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H225" t="s">
         <v>1075</v>
@@ -46217,10 +46217,10 @@
         <v>1048</v>
       </c>
       <c r="F226">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G226">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H226" t="s">
         <v>769</v>
@@ -46402,10 +46402,10 @@
         <v>1048</v>
       </c>
       <c r="F227">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G227">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H227" t="s">
         <v>769</v>
@@ -46587,10 +46587,10 @@
         <v>1048</v>
       </c>
       <c r="F228">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G228">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H228" t="s">
         <v>655</v>
@@ -46772,10 +46772,10 @@
         <v>1048</v>
       </c>
       <c r="F229">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G229">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H229" t="s">
         <v>655</v>
@@ -46957,10 +46957,10 @@
         <v>1048</v>
       </c>
       <c r="F230">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G230">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H230" t="s">
         <v>1084</v>
@@ -47142,10 +47142,10 @@
         <v>1048</v>
       </c>
       <c r="F231">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G231">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H231" t="s">
         <v>780</v>
@@ -47327,10 +47327,10 @@
         <v>1048</v>
       </c>
       <c r="F232">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G232">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H232" t="s">
         <v>780</v>
@@ -47512,10 +47512,10 @@
         <v>1048</v>
       </c>
       <c r="F233">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G233">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H233" t="s">
         <v>1090</v>
@@ -47697,10 +47697,10 @@
         <v>1048</v>
       </c>
       <c r="F234">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G234">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H234" t="s">
         <v>1094</v>
@@ -47882,10 +47882,10 @@
         <v>1048</v>
       </c>
       <c r="F235">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G235">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H235" t="s">
         <v>821</v>
@@ -48067,10 +48067,10 @@
         <v>1048</v>
       </c>
       <c r="F236">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G236">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H236" t="s">
         <v>364</v>
@@ -48252,10 +48252,10 @@
         <v>1048</v>
       </c>
       <c r="F237">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G237">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H237" t="s">
         <v>686</v>
@@ -48437,10 +48437,10 @@
         <v>1048</v>
       </c>
       <c r="F238">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G238">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H238" t="s">
         <v>1070</v>
@@ -48622,10 +48622,10 @@
         <v>1048</v>
       </c>
       <c r="F239">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G239">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H239" t="s">
         <v>686</v>
@@ -48807,10 +48807,10 @@
         <v>1048</v>
       </c>
       <c r="F240">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G240">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H240" t="s">
         <v>1103</v>
@@ -48992,10 +48992,10 @@
         <v>1048</v>
       </c>
       <c r="F241">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G241">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H241" t="s">
         <v>391</v>
@@ -49177,10 +49177,10 @@
         <v>1048</v>
       </c>
       <c r="F242">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G242">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H242" t="s">
         <v>1110</v>
@@ -49362,10 +49362,10 @@
         <v>1048</v>
       </c>
       <c r="F243">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G243">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H243" t="s">
         <v>1117</v>
@@ -49547,10 +49547,10 @@
         <v>1048</v>
       </c>
       <c r="F244">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G244">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H244" t="s">
         <v>1125</v>
@@ -49732,10 +49732,10 @@
         <v>1048</v>
       </c>
       <c r="F245">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G245">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H245" t="s">
         <v>671</v>
@@ -49917,10 +49917,10 @@
         <v>836</v>
       </c>
       <c r="F246">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G246">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H246" t="s">
         <v>413</v>
@@ -50102,10 +50102,10 @@
         <v>1048</v>
       </c>
       <c r="F247">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G247">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H247" t="s">
         <v>1136</v>
@@ -50287,10 +50287,10 @@
         <v>836</v>
       </c>
       <c r="F248">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G248">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H248" t="s">
         <v>671</v>
@@ -50472,10 +50472,10 @@
         <v>1048</v>
       </c>
       <c r="F249">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G249">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H249" t="s">
         <v>1136</v>
@@ -50657,10 +50657,10 @@
         <v>1048</v>
       </c>
       <c r="F250">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G250">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H250" t="s">
         <v>1143</v>
@@ -50842,10 +50842,10 @@
         <v>1048</v>
       </c>
       <c r="F251">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G251">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H251" t="s">
         <v>1143</v>
@@ -51027,10 +51027,10 @@
         <v>1048</v>
       </c>
       <c r="F252">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G252">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H252" t="s">
         <v>671</v>
@@ -51212,10 +51212,10 @@
         <v>1048</v>
       </c>
       <c r="F253">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G253">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H253" t="s">
         <v>1156</v>
@@ -51397,10 +51397,10 @@
         <v>1048</v>
       </c>
       <c r="F254">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G254">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H254" t="s">
         <v>1163</v>
@@ -51582,10 +51582,10 @@
         <v>1048</v>
       </c>
       <c r="F255">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G255">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H255" t="s">
         <v>364</v>
@@ -51767,10 +51767,10 @@
         <v>1048</v>
       </c>
       <c r="F256">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G256">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H256" t="s">
         <v>240</v>
@@ -51952,10 +51952,10 @@
         <v>1048</v>
       </c>
       <c r="F257">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G257">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H257" t="s">
         <v>1163</v>
@@ -52137,10 +52137,10 @@
         <v>1048</v>
       </c>
       <c r="F258">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G258">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H258" t="s">
         <v>637</v>
@@ -52322,10 +52322,10 @@
         <v>836</v>
       </c>
       <c r="F259">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G259">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H259" t="s">
         <v>90</v>
@@ -52507,10 +52507,10 @@
         <v>1048</v>
       </c>
       <c r="F260">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G260">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H260" t="s">
         <v>1173</v>
@@ -52692,10 +52692,10 @@
         <v>1048</v>
       </c>
       <c r="F261">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G261">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H261" t="s">
         <v>217</v>
@@ -52877,10 +52877,10 @@
         <v>1048</v>
       </c>
       <c r="F262">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G262">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H262" t="s">
         <v>1173</v>
@@ -53062,10 +53062,10 @@
         <v>1048</v>
       </c>
       <c r="F263">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G263">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H263" t="s">
         <v>637</v>
@@ -53247,10 +53247,10 @@
         <v>1048</v>
       </c>
       <c r="F264">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G264">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H264" t="s">
         <v>1182</v>
@@ -53432,10 +53432,10 @@
         <v>1048</v>
       </c>
       <c r="F265">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G265">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H265" t="s">
         <v>1186</v>
@@ -53617,10 +53617,10 @@
         <v>1048</v>
       </c>
       <c r="F266">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G266">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H266" t="s">
         <v>1191</v>
@@ -53802,10 +53802,10 @@
         <v>836</v>
       </c>
       <c r="F267">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G267">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H267" t="s">
         <v>1196</v>
@@ -53987,10 +53987,10 @@
         <v>836</v>
       </c>
       <c r="F268">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G268">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H268" t="s">
         <v>1196</v>
@@ -54172,10 +54172,10 @@
         <v>1048</v>
       </c>
       <c r="F269">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G269">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H269" t="s">
         <v>1201</v>
@@ -54357,10 +54357,10 @@
         <v>1048</v>
       </c>
       <c r="F270">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G270">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H270" t="s">
         <v>1206</v>
@@ -54542,10 +54542,10 @@
         <v>1048</v>
       </c>
       <c r="F271">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G271">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H271" t="s">
         <v>1212</v>
@@ -54727,10 +54727,10 @@
         <v>1048</v>
       </c>
       <c r="F272">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G272">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H272" t="s">
         <v>612</v>
@@ -54912,10 +54912,10 @@
         <v>1048</v>
       </c>
       <c r="F273">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G273">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H273" t="s">
         <v>1217</v>
@@ -55097,10 +55097,10 @@
         <v>1048</v>
       </c>
       <c r="F274">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G274">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H274" t="s">
         <v>1217</v>
@@ -55282,10 +55282,10 @@
         <v>1048</v>
       </c>
       <c r="F275">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G275">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H275" t="s">
         <v>1221</v>
@@ -55467,10 +55467,10 @@
         <v>1048</v>
       </c>
       <c r="F276">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G276">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H276" t="s">
         <v>1227</v>
@@ -55652,10 +55652,10 @@
         <v>836</v>
       </c>
       <c r="F277">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G277">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H277" t="s">
         <v>1231</v>
@@ -55837,10 +55837,10 @@
         <v>1048</v>
       </c>
       <c r="F278">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G278">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H278" t="s">
         <v>1234</v>
@@ -56022,10 +56022,10 @@
         <v>1048</v>
       </c>
       <c r="F279">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G279">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H279" t="s">
         <v>217</v>
@@ -56207,10 +56207,10 @@
         <v>1048</v>
       </c>
       <c r="F280">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G280">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H280" t="s">
         <v>109</v>
@@ -56392,10 +56392,10 @@
         <v>1048</v>
       </c>
       <c r="F281">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G281">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H281" t="s">
         <v>1059</v>
@@ -56577,10 +56577,10 @@
         <v>1048</v>
       </c>
       <c r="F282">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G282">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H282" t="s">
         <v>262</v>
@@ -56762,10 +56762,10 @@
         <v>1243</v>
       </c>
       <c r="F283">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G283">
-        <v>-20</v>
+        <v>-18</v>
       </c>
       <c r="H283" t="s">
         <v>443</v>
@@ -56947,10 +56947,10 @@
         <v>836</v>
       </c>
       <c r="F284">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G284">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H284" t="s">
         <v>631</v>
@@ -57132,10 +57132,10 @@
         <v>836</v>
       </c>
       <c r="F285">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G285">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H285" t="s">
         <v>1251</v>
@@ -57317,10 +57317,10 @@
         <v>836</v>
       </c>
       <c r="F286">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G286">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H286" t="s">
         <v>1251</v>
@@ -57502,10 +57502,10 @@
         <v>836</v>
       </c>
       <c r="F287">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G287">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H287" t="s">
         <v>1257</v>
@@ -57687,10 +57687,10 @@
         <v>1048</v>
       </c>
       <c r="F288">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G288">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H288" t="s">
         <v>889</v>
@@ -57872,10 +57872,10 @@
         <v>836</v>
       </c>
       <c r="F289">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G289">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H289" t="s">
         <v>724</v>
@@ -58057,10 +58057,10 @@
         <v>836</v>
       </c>
       <c r="F290">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G290">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H290" t="s">
         <v>1262</v>
@@ -58242,10 +58242,10 @@
         <v>836</v>
       </c>
       <c r="F291">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G291">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H291" t="s">
         <v>964</v>
@@ -58427,10 +58427,10 @@
         <v>836</v>
       </c>
       <c r="F292">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G292">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H292" t="s">
         <v>1269</v>
@@ -58612,10 +58612,10 @@
         <v>836</v>
       </c>
       <c r="F293">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G293">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H293" t="s">
         <v>732</v>
@@ -58797,10 +58797,10 @@
         <v>836</v>
       </c>
       <c r="F294">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G294">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H294" t="s">
         <v>1275</v>
@@ -58982,10 +58982,10 @@
         <v>836</v>
       </c>
       <c r="F295">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G295">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H295" t="s">
         <v>90</v>
@@ -59167,10 +59167,10 @@
         <v>1290</v>
       </c>
       <c r="F296">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G296">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H296" t="s">
         <v>1291</v>
@@ -59352,10 +59352,10 @@
         <v>1297</v>
       </c>
       <c r="F297">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G297">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H297" t="s">
         <v>1298</v>
@@ -59537,10 +59537,10 @@
         <v>153</v>
       </c>
       <c r="F298">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G298">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H298" t="s">
         <v>1304</v>
@@ -59722,10 +59722,10 @@
         <v>204</v>
       </c>
       <c r="F299">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G299">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H299" t="s">
         <v>1307</v>
@@ -59907,10 +59907,10 @@
         <v>247</v>
       </c>
       <c r="F300">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G300">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H300" t="s">
         <v>212</v>
@@ -60092,10 +60092,10 @@
         <v>273</v>
       </c>
       <c r="F301">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G301">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H301" t="s">
         <v>1291</v>
@@ -60277,10 +60277,10 @@
         <v>274</v>
       </c>
       <c r="F302">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G302">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H302" t="s">
         <v>1307</v>
@@ -60462,10 +60462,10 @@
         <v>329</v>
       </c>
       <c r="F303">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G303">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H303" t="s">
         <v>1291</v>
@@ -60647,7 +60647,7 @@
         <v>355</v>
       </c>
       <c r="F304">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G304">
         <v>2</v>
@@ -60832,7 +60832,7 @@
         <v>355</v>
       </c>
       <c r="F305">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G305">
         <v>2</v>
@@ -61017,10 +61017,10 @@
         <v>420</v>
       </c>
       <c r="F306">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G306">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H306" t="s">
         <v>1307</v>
@@ -61202,10 +61202,10 @@
         <v>551</v>
       </c>
       <c r="F307">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G307">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H307" t="s">
         <v>368</v>
@@ -61387,10 +61387,10 @@
         <v>654</v>
       </c>
       <c r="F308">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G308">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H308" t="s">
         <v>1307</v>
@@ -61572,10 +61572,10 @@
         <v>751</v>
       </c>
       <c r="F309">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G309">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H309" t="s">
         <v>856</v>
@@ -61757,10 +61757,10 @@
         <v>751</v>
       </c>
       <c r="F310">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G310">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H310" t="s">
         <v>1307</v>
@@ -61942,10 +61942,10 @@
         <v>751</v>
       </c>
       <c r="F311">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G311">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H311" t="s">
         <v>934</v>
@@ -62127,10 +62127,10 @@
         <v>836</v>
       </c>
       <c r="F312">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G312">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H312" t="s">
         <v>226</v>
@@ -62312,10 +62312,10 @@
         <v>836</v>
       </c>
       <c r="F313">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G313">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H313" t="s">
         <v>249</v>
@@ -62497,10 +62497,10 @@
         <v>836</v>
       </c>
       <c r="F314">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G314">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H314" t="s">
         <v>249</v>
@@ -62682,10 +62682,10 @@
         <v>836</v>
       </c>
       <c r="F315">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G315">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H315" t="s">
         <v>249</v>
@@ -62867,10 +62867,10 @@
         <v>836</v>
       </c>
       <c r="F316">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G316">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H316" t="s">
         <v>1022</v>
@@ -63052,10 +63052,10 @@
         <v>836</v>
       </c>
       <c r="F317">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G317">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H317" t="s">
         <v>1022</v>
@@ -63237,10 +63237,10 @@
         <v>1048</v>
       </c>
       <c r="F318">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G318">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H318" t="s">
         <v>671</v>
@@ -63422,10 +63422,10 @@
         <v>1048</v>
       </c>
       <c r="F319">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G319">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H319" t="s">
         <v>671</v>
@@ -63607,10 +63607,10 @@
         <v>836</v>
       </c>
       <c r="F320">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G320">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H320" t="s">
         <v>1341</v>
@@ -63792,10 +63792,10 @@
         <v>836</v>
       </c>
       <c r="F321">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G321">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H321" t="s">
         <v>1341</v>
@@ -63977,10 +63977,10 @@
         <v>1290</v>
       </c>
       <c r="F322">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="G322">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H322" t="s">
         <v>1350</v>
@@ -64162,10 +64162,10 @@
         <v>231</v>
       </c>
       <c r="F323">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G323">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H323" t="s">
         <v>1350</v>
@@ -64347,10 +64347,10 @@
         <v>304</v>
       </c>
       <c r="F324">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G324">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H324" t="s">
         <v>1350</v>
@@ -64532,10 +64532,10 @@
         <v>329</v>
       </c>
       <c r="F325">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G325">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H325" t="s">
         <v>663</v>
@@ -64717,10 +64717,10 @@
         <v>330</v>
       </c>
       <c r="F326">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G326">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H326" t="s">
         <v>1350</v>
@@ -64902,10 +64902,10 @@
         <v>836</v>
       </c>
       <c r="F327">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G327">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H327" t="s">
         <v>1350</v>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 24/08/2026 18:18:13
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{046E8D92-0F41-4B5A-B08D-EA32CC001015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C523C1AE-FB35-4A5D-99F6-A4C649316FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="15375" windowHeight="8325" xr2:uid="{3A8E4734-8B72-4AAA-B9B5-B0D6667DB0DF}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="15375" windowHeight="8325" xr2:uid="{3BA89D0F-47AE-4B8D-934C-F8D92D39F491}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -4348,7 +4348,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81724EAB-C57F-4AB3-8AE8-486E4EE9B127}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61373715-BD06-4DC6-8720-58A366F57F07}">
   <dimension ref="A1:BI304"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>

<commit_message>
Actualización automática ERP - Pedidos Pendientes - 26/08/2026 15:55:40
</commit_message>
<xml_diff>
--- a/Data_ERP/Pedidos Pendientes.xlsx
+++ b/Data_ERP/Pedidos Pendientes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sistema_Logistico_Peirano\Data_ERP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2ABBD9EA-B728-4E28-88A9-F05424D3CFA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0ECB7C5F-AEFE-4E93-9FA9-F50E6C963036}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24885" yWindow="3735" windowWidth="15375" windowHeight="8325" xr2:uid="{8039B828-C670-4A82-83EA-CFE0E62A6AA4}"/>
+    <workbookView xWindow="24885" yWindow="3735" windowWidth="15375" windowHeight="8325" xr2:uid="{7B3D96FE-D622-476E-88A9-F1D1D14CC410}"/>
   </bookViews>
   <sheets>
     <sheet name="pedidos pendientes" sheetId="1" r:id="rId1"/>
@@ -5119,7 +5119,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8034BF66-AD46-4CC5-BBBB-CCF6F509AA3B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F8F4CAB-B23B-445B-8A4B-6D2D22340AF5}">
   <dimension ref="A1:BI380"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <sheetData>

</xml_diff>